<commit_message>
cab 10 19.05.2026 12:09
</commit_message>
<xml_diff>
--- a/sample_data.xlsx
+++ b/sample_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason\Projects\load_configurator_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AEDAA37-146F-4FA3-A823-4BE832B28CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EDED954-948E-4AA4-819F-346961E26BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-43476" yWindow="1188" windowWidth="17280" windowHeight="8880" xr2:uid="{A1139CED-2EED-461D-8A45-C2AEED3E8BCB}"/>
+    <workbookView xWindow="-46188" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A1139CED-2EED-461D-8A45-C2AEED3E8BCB}"/>
   </bookViews>
   <sheets>
     <sheet name="sample_data1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="32">
   <si>
     <t>LENGTH</t>
   </si>
@@ -104,6 +104,18 @@
   </si>
   <si>
     <t>DE33GC</t>
+  </si>
+  <si>
+    <t>DE250E0</t>
+  </si>
+  <si>
+    <t>DE660E0</t>
+  </si>
+  <si>
+    <t>DE16E0</t>
+  </si>
+  <si>
+    <t>DE330E0</t>
   </si>
 </sst>
 </file>
@@ -255,7 +267,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -441,20 +453,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="26">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -606,19 +606,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -658,135 +645,10 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -836,7 +698,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -847,134 +709,29 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="2" fontId="0" fillId="33" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="33" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="33" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="33" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="34" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="34" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="34" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="34" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="34" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="34" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="35" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="35" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="35" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="35" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1351,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F99A702-F2DD-4857-BE6B-40AE175852D3}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.88671875" bestFit="1" customWidth="1"/>
@@ -1408,7 +1165,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1426,559 +1183,856 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>1.1200000000000001</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1.62</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="5">
         <v>1.3580000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="6">
-        <v>3.38</v>
-      </c>
-      <c r="C6" s="6">
-        <v>1.17</v>
-      </c>
-      <c r="D6" s="6">
-        <v>1.85</v>
-      </c>
-      <c r="E6" s="10">
-        <v>1.881</v>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1.62</v>
+      </c>
+      <c r="E6" s="5">
+        <v>1.3580000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1.62</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1.3580000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1.62</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1.3580000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B9" s="4">
         <v>2.77</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C9" s="4">
         <v>1.1200000000000001</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D9" s="4">
         <v>1.63</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E9" s="5">
         <v>1.51</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="4">
+        <v>2.77</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1.63</v>
+      </c>
+      <c r="E10" s="5">
+        <v>1.51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B11" s="4">
         <v>2.8</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C11" s="4">
         <v>1.05</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D11" s="4">
         <v>1.68</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E11" s="5">
         <v>1.196</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B12" s="4">
         <v>2.8</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C12" s="4">
         <v>1.05</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D12" s="4">
         <v>1.68</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E12" s="5">
         <v>1.196</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="6">
-        <v>3.38</v>
-      </c>
-      <c r="C10" s="6">
-        <v>1.17</v>
-      </c>
-      <c r="D10" s="6">
-        <v>1.85</v>
-      </c>
-      <c r="E10" s="10">
-        <v>1.881</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="5">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="C11" s="5">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="D11" s="5">
-        <v>1.62</v>
-      </c>
-      <c r="E11" s="13">
-        <v>1.3580000000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="6">
-        <v>3.38</v>
-      </c>
-      <c r="C12" s="6">
-        <v>1.17</v>
-      </c>
-      <c r="D12" s="6">
-        <v>1.85</v>
-      </c>
-      <c r="E12" s="14">
-        <v>1.881</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="7">
-        <v>2.77</v>
-      </c>
-      <c r="C13" s="7">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="D13" s="7">
+        <v>19</v>
+      </c>
+      <c r="B13" s="4">
+        <v>2.8</v>
+      </c>
+      <c r="C13" s="4">
+        <v>1.05</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1.68</v>
+      </c>
+      <c r="E13" s="5">
+        <v>1.196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="4">
+        <v>2.8</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1.05</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1.68</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1.196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C15" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D15" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E15" s="5">
+        <v>1.881</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1.881</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C17" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E17" s="5">
+        <v>1.881</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="4">
+        <v>2.6619999999999999</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1.1120000000000001</v>
+      </c>
+      <c r="D18" s="4">
+        <v>1.766</v>
+      </c>
+      <c r="E18" s="5">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4">
+        <v>2.6619999999999999</v>
+      </c>
+      <c r="C19" s="4">
+        <v>1.1120000000000001</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1.766</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C20" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E20" s="5">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C21" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D21" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E21" s="5">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C22" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D22" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E22" s="5">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4">
+        <v>3.38</v>
+      </c>
+      <c r="C23" s="4">
+        <v>1.17</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1.85</v>
+      </c>
+      <c r="E23" s="5">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="4">
+        <v>4.03</v>
+      </c>
+      <c r="C24" s="4">
+        <v>1.46</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2.19</v>
+      </c>
+      <c r="E24" s="5">
+        <v>2.782</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="4">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="C25" s="4">
         <v>1.63</v>
       </c>
-      <c r="E13" s="15">
-        <v>1.51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="8">
-        <v>2.8</v>
-      </c>
-      <c r="C14" s="8">
-        <v>1.05</v>
-      </c>
-      <c r="D14" s="8">
-        <v>1.68</v>
-      </c>
-      <c r="E14" s="16">
-        <v>1.196</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="8">
-        <v>2.8</v>
-      </c>
-      <c r="C15" s="8">
-        <v>1.05</v>
-      </c>
-      <c r="D15" s="8">
-        <v>1.68</v>
-      </c>
-      <c r="E15" s="16">
-        <v>1.196</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="6">
-        <v>3.38</v>
-      </c>
-      <c r="C16" s="6">
-        <v>1.17</v>
-      </c>
-      <c r="D16" s="6">
-        <v>1.85</v>
-      </c>
-      <c r="E16" s="14">
-        <v>1.88</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="18">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="C17" s="18">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="D17" s="18">
-        <v>1.62</v>
-      </c>
-      <c r="E17" s="19">
-        <v>1.3580000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="21">
-        <v>3.38</v>
-      </c>
-      <c r="C18" s="21">
-        <v>1.17</v>
-      </c>
-      <c r="D18" s="21">
-        <v>1.85</v>
-      </c>
-      <c r="E18" s="22">
-        <v>1.88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="24">
-        <v>4</v>
-      </c>
-      <c r="C19" s="24">
+      <c r="D25" s="4">
+        <v>2.36</v>
+      </c>
+      <c r="E25" s="5">
+        <v>3.8079999999999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1.63</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2.36</v>
+      </c>
+      <c r="E26" s="5">
+        <v>3.8079999999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C27" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D27" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E27" s="5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C28" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D28" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E28" s="5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C29" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E29" s="5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C30" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D30" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E30" s="5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" s="4">
+        <v>5.5720000000000001</v>
+      </c>
+      <c r="C31" s="6">
+        <v>2.17</v>
+      </c>
+      <c r="D31" s="4">
+        <v>2.3980000000000001</v>
+      </c>
+      <c r="E31" s="5">
+        <v>6.69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="7">
+        <v>5.5720000000000001</v>
+      </c>
+      <c r="C32" s="8">
+        <v>2.17</v>
+      </c>
+      <c r="D32" s="7">
+        <v>2.3980000000000001</v>
+      </c>
+      <c r="E32" s="9">
+        <v>6.69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4">
+        <v>5.32</v>
+      </c>
+      <c r="C33" s="4">
+        <v>1.92</v>
+      </c>
+      <c r="D33" s="4">
+        <v>2.29</v>
+      </c>
+      <c r="E33" s="5">
+        <v>5.952</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="10">
+        <v>2</v>
+      </c>
+      <c r="C34" s="10">
+        <v>0.92</v>
+      </c>
+      <c r="D34" s="10">
+        <v>1.44</v>
+      </c>
+      <c r="E34" s="11">
+        <v>0.83799999999999997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2</v>
+      </c>
+      <c r="C35" s="4">
+        <v>0.92</v>
+      </c>
+      <c r="D35" s="4">
+        <v>1.44</v>
+      </c>
+      <c r="E35" s="5">
+        <v>0.83799999999999997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B36" s="4">
+        <v>2</v>
+      </c>
+      <c r="C36" s="4">
+        <v>0.92</v>
+      </c>
+      <c r="D36" s="4">
+        <v>1.44</v>
+      </c>
+      <c r="E36" s="5">
+        <v>0.83799999999999997</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" s="4">
+        <v>2</v>
+      </c>
+      <c r="C37" s="4">
+        <v>0.92</v>
+      </c>
+      <c r="D37" s="4">
+        <v>1.44</v>
+      </c>
+      <c r="E37" s="5">
+        <v>0.83799999999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B38" s="4">
+        <v>2</v>
+      </c>
+      <c r="C38" s="4">
+        <v>0.92</v>
+      </c>
+      <c r="D38" s="4">
+        <v>1.44</v>
+      </c>
+      <c r="E38" s="5">
+        <v>0.83799999999999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="4">
+        <v>4.93</v>
+      </c>
+      <c r="C39" s="4">
+        <v>1.66</v>
+      </c>
+      <c r="D39" s="4">
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="E39" s="5">
+        <v>4.7069999999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B40" s="4">
+        <v>2</v>
+      </c>
+      <c r="C40" s="4">
+        <v>0.92</v>
+      </c>
+      <c r="D40" s="4">
+        <v>1.44</v>
+      </c>
+      <c r="E40" s="5">
+        <v>0.83699999999999997</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="C41" s="4">
+        <v>0.62</v>
+      </c>
+      <c r="D41" s="4">
+        <v>1.115</v>
+      </c>
+      <c r="E41" s="5">
+        <v>0.44700000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="C42" s="4">
+        <v>0.62</v>
+      </c>
+      <c r="D42" s="4">
+        <v>1.115</v>
+      </c>
+      <c r="E42" s="5">
+        <v>0.44700000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B43" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C43" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D43" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E43" s="5">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C44" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D44" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E44" s="5">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B45" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C45" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D45" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E45" s="5">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B46" s="4">
+        <v>4.03</v>
+      </c>
+      <c r="C46" s="4">
         <v>1.46</v>
       </c>
-      <c r="D19" s="24">
-        <v>2.12</v>
-      </c>
-      <c r="E19" s="25">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
+      <c r="D46" s="4">
+        <v>2.19</v>
+      </c>
+      <c r="E46" s="5">
+        <v>2.782</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B47" s="4">
+        <v>3.988</v>
+      </c>
+      <c r="C47" s="4">
+        <v>1.2070000000000001</v>
+      </c>
+      <c r="D47" s="4">
+        <v>1.867</v>
+      </c>
+      <c r="E47" s="5">
+        <v>2.8540000000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48" s="4">
+        <v>4.93</v>
+      </c>
+      <c r="C48" s="4">
+        <v>1.66</v>
+      </c>
+      <c r="D48" s="4">
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="E48" s="5">
+        <v>4.7069999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B49" s="4">
+        <v>4.93</v>
+      </c>
+      <c r="C49" s="4">
+        <v>1.66</v>
+      </c>
+      <c r="D49" s="4">
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="E49" s="5">
+        <v>4.7069999999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B50" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C50" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D50" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E50" s="5">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B51" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C51" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D51" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E51" s="5">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B52" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C52" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D52" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E52" s="5">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="27">
+      <c r="B53" s="4">
+        <v>2.33</v>
+      </c>
+      <c r="C53" s="4">
         <v>0.96</v>
       </c>
-      <c r="C20" s="27">
+      <c r="D53" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="E53" s="5">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="4">
         <v>2.33</v>
       </c>
-      <c r="D20" s="27">
+      <c r="C54" s="4">
+        <v>0.96</v>
+      </c>
+      <c r="D54" s="4">
         <v>1.5</v>
       </c>
-      <c r="E20" s="28">
+      <c r="E54" s="5">
         <v>0.98</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="27">
-        <v>0.96</v>
-      </c>
-      <c r="C21" s="27">
-        <v>2.33</v>
-      </c>
-      <c r="D21" s="27">
-        <v>1.5</v>
-      </c>
-      <c r="E21" s="28">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="27">
-        <v>0.96</v>
-      </c>
-      <c r="C22" s="27">
-        <v>2.33</v>
-      </c>
-      <c r="D22" s="27">
-        <v>1.5</v>
-      </c>
-      <c r="E22" s="28">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23" s="27">
-        <v>0.96</v>
-      </c>
-      <c r="C23" s="27">
-        <v>2.33</v>
-      </c>
-      <c r="D23" s="27">
-        <v>1.5</v>
-      </c>
-      <c r="E23" s="28">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="21">
-        <v>4.93</v>
-      </c>
-      <c r="C24" s="21">
-        <v>1.66</v>
-      </c>
-      <c r="D24" s="21">
-        <v>2.3199999999999998</v>
-      </c>
-      <c r="E24" s="22">
-        <v>4.7069999999999999</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="18">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="C25" s="18">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="D25" s="18">
-        <v>1.62</v>
-      </c>
-      <c r="E25" s="19">
-        <v>1.3580000000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="21">
-        <v>3.38</v>
-      </c>
-      <c r="C26" s="21">
-        <v>1.17</v>
-      </c>
-      <c r="D26" s="21">
-        <v>1.85</v>
-      </c>
-      <c r="E26" s="22">
-        <v>1.88</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="30">
-        <v>5.5720000000000001</v>
-      </c>
-      <c r="C27" s="30">
-        <v>2.17</v>
-      </c>
-      <c r="D27" s="30">
-        <v>2.3980000000000001</v>
-      </c>
-      <c r="E27" s="31">
-        <v>6.69</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="33">
-        <v>4.7699999999999996</v>
-      </c>
-      <c r="C28" s="33">
-        <v>1.63</v>
-      </c>
-      <c r="D28" s="33">
-        <v>2.36</v>
-      </c>
-      <c r="E28" s="34">
-        <v>3.8079999999999998</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="35"/>
-      <c r="B29" s="36"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="36">
-        <v>4.7699999999999996</v>
-      </c>
-      <c r="C30" s="36">
-        <v>1.63</v>
-      </c>
-      <c r="D30" s="36">
-        <v>2.36</v>
-      </c>
-      <c r="E30" s="37">
-        <v>3.8079999999999998</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="35"/>
-      <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="37"/>
-    </row>
-    <row r="32" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" s="39">
-        <v>2.33</v>
-      </c>
-      <c r="C32" s="39">
-        <v>0.96</v>
-      </c>
-      <c r="D32" s="39">
-        <v>1.5</v>
-      </c>
-      <c r="E32" s="40">
-        <v>0.877</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="B33" s="42">
-        <v>2</v>
-      </c>
-      <c r="C33" s="42">
-        <v>0.92</v>
-      </c>
-      <c r="D33" s="42">
-        <v>1.44</v>
-      </c>
-      <c r="E33" s="43">
-        <v>0.83799999999999997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="B34" s="45">
-        <v>2</v>
-      </c>
-      <c r="C34" s="45">
-        <v>0.92</v>
-      </c>
-      <c r="D34" s="45">
-        <v>1.44</v>
-      </c>
-      <c r="E34" s="46">
-        <v>0.83799999999999997</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="B35" s="45">
-        <v>2</v>
-      </c>
-      <c r="C35" s="45">
-        <v>0.92</v>
-      </c>
-      <c r="D35" s="45">
-        <v>1.44</v>
-      </c>
-      <c r="E35" s="46">
-        <v>0.83799999999999997</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="B36" s="45">
-        <v>2</v>
-      </c>
-      <c r="C36" s="45">
-        <v>0.92</v>
-      </c>
-      <c r="D36" s="45">
-        <v>1.44</v>
-      </c>
-      <c r="E36" s="46">
-        <v>0.83799999999999997</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="B37" s="39">
-        <v>2.33</v>
-      </c>
-      <c r="C37" s="39">
-        <v>0.96</v>
-      </c>
-      <c r="D37" s="39">
-        <v>1.5</v>
-      </c>
-      <c r="E37" s="40">
-        <v>0.877</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>